<commit_message>
docs: balance de comida en Recursos.xlsx, fichas, GDD 3.35 y documentos técnicos
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SJTyjZex75AFX3j4vFf7i6
</commit_message>
<xml_diff>
--- a/docs/Recursos.xlsx
+++ b/docs/Recursos.xlsx
@@ -1705,7 +1705,7 @@
         <v>5</v>
       </c>
       <c r="G2" t="n">
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -1756,7 +1756,7 @@
         <v>5</v>
       </c>
       <c r="G3" t="n">
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -1807,7 +1807,7 @@
         <v>5</v>
       </c>
       <c r="G4" t="n">
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -1858,7 +1858,7 @@
         <v>5</v>
       </c>
       <c r="G5" t="n">
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -1909,7 +1909,7 @@
         <v>5</v>
       </c>
       <c r="G6" t="n">
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -1960,7 +1960,7 @@
         <v>5</v>
       </c>
       <c r="G7" t="n">
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -2011,7 +2011,7 @@
         <v>5</v>
       </c>
       <c r="G8" t="n">
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -2051,18 +2051,18 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>densidad de fauna (Excel: venado)</t>
+          <t>densidad de fauna (reemplaza el venado 15 del Excel por el balance del 2026-09-21; el venado 15 sigue en la hoja Relacion)</t>
         </is>
       </c>
       <c r="F9" t="n">
         <v>7</v>
       </c>
       <c r="G9" t="n">
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -2113,7 +2113,7 @@
         <v>7</v>
       </c>
       <c r="G10" t="n">
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -2153,7 +2153,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -2164,7 +2164,7 @@
         <v>7</v>
       </c>
       <c r="G11" t="n">
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -2204,7 +2204,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -2215,7 +2215,7 @@
         <v>7</v>
       </c>
       <c r="G12" t="n">
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -2414,7 +2414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" style="2" min="1" max="1"/>
@@ -2492,7 +2492,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>20</v>
+        <v>150</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -2512,7 +2512,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -2536,7 +2536,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>unidades por recurso (comida: 2000)</t>
+          <t>unidades por recurso (comida: 10000)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -2552,7 +2552,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2000</v>
+        <v>10000</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -2662,6 +2662,46 @@
       <c r="D12" t="inlineStr">
         <is>
           <t>Ciudad.TIPOS_POBLACION</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Meta de comida por recolector</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>comida por hora a densidad media (5 propio + 2,5 de medio acarreador)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Recoleccion.gd, balance del 2026-09-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Comida del avatar</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>5</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>comida por hora a nivel 1</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Ciudad.Avatar.tasa_hambre</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: caza 14 y frutos 8 en Recursos.xlsx, fichas, GDD 3.36 y documentos técnicos
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SJTyjZex75AFX3j4vFf7i6
</commit_message>
<xml_diff>
--- a/docs/Recursos.xlsx
+++ b/docs/Recursos.xlsx
@@ -2051,11 +2051,11 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>densidad de fauna (reemplaza el venado 15 del Excel por el balance del 2026-09-21; el venado 15 sigue en la hoja Relacion)</t>
+          <t>densidad de fauna (decisión del usuario, 2026-09-21: 14; el primer balance del día dejó 10; reemplaza el venado 15 del Excel, que sigue en la hoja Relacion)</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -2102,11 +2102,11 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>densidad frutal (Excel: columna Árbol (obj), Comida 5; interpretada como frutos)</t>
+          <t>densidad frutal (originalmente interpretada de la columna Árbol (obj) del Excel, Comida 5; cambiada a 8 por decisión del usuario, 2026-09-21)</t>
         </is>
       </c>
       <c r="F10" t="n">
@@ -2676,12 +2676,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>comida por hora a densidad media (5 propio + 2,5 de medio acarreador)</t>
+          <t>comida por hora como mínimo por recolector (5 propio + 2,5 de medio acarreador); cumplida con margen: caza + frutos ≈ 10,0/h y pesca ≈ 8,6/h medidos en el mundo actual (semilla 12345)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Recoleccion.gd, balance del 2026-09-21</t>
+          <t>Recoleccion.gd, balance del 2026-09-21 (caza 14 y frutos 8 por decisión del usuario)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: pesca por tamaño y profundidad en Recursos.xlsx, fichas, GDD 3.37 y documentos técnicos
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SJTyjZex75AFX3j4vFf7i6
</commit_message>
<xml_diff>
--- a/docs/Recursos.xlsx
+++ b/docs/Recursos.xlsx
@@ -2153,11 +2153,11 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>densidad de peces</t>
+          <t>densidad de peces ponderada por profundidad (×0,5 en agua somera a ×1,5 en la más profunda) × escala por tamaño del agua (celdas conectadas / 450, mín 0,4, máx 1,5); decisión del usuario, 2026-09-21: base 17 (antes 12) para compensar el descuento por profundidad</t>
         </is>
       </c>
       <c r="F11" t="n">
@@ -2208,7 +2208,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>densidad de algas</t>
+          <t>densidad de algas × la misma escala por tamaño del agua</t>
         </is>
       </c>
       <c r="F12" t="n">
@@ -2414,7 +2414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" style="2" min="1" max="1"/>
@@ -2705,6 +2705,66 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Agua de referencia (pesca)</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>450</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>celdas de agua conectada dentro del radio 25 que dan escala 1,0 (mediana del mundo actual)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Recoleccion.AGUA_REFERENCIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Escala de agua mínima</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>multiplicador de la pesca y las algas con poca agua</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Recoleccion.ESCALA_AGUA_MIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Escala de agua máxima</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>multiplicador de la pesca y las algas con mucha agua</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Recoleccion.ESCALA_AGUA_MAX</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: HUD con promedio de 10 h en /h y caza 17 / frutos 10
Recurso.tasa_neta_promedio (ventana de 10 h) alimenta el HUD y recurso_critico();
la lista muestra /h en vez de /tick. Caza y recolección sube de 14/8 a 17/10
(~12,2 comida/h de media frente a ~8,6 de la pesca). Docs: GDD 3.38, Excel, fichas, PoC 5 y 6.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SJTyjZex75AFX3j4vFf7i6
</commit_message>
<xml_diff>
--- a/docs/Recursos.xlsx
+++ b/docs/Recursos.xlsx
@@ -2051,11 +2051,11 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>densidad de fauna (decisión del usuario, 2026-09-21: 14; el primer balance del día dejó 10; reemplaza el venado 15 del Excel, que sigue en la hoja Relacion)</t>
+          <t>densidad de fauna (decisión del usuario, 2026-09-21: 17; el primer balance del día dejó 10 y el segundo 14; reemplaza el venado 15 del Excel, que sigue en la hoja Relacion)</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -2102,11 +2102,11 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>densidad frutal (originalmente interpretada de la columna Árbol (obj) del Excel, Comida 5; cambiada a 8 por decisión del usuario, 2026-09-21)</t>
+          <t>densidad frutal (originalmente interpretada de la columna Árbol (obj) del Excel, Comida 5; cambiada a 8 y luego a 10 por decisión del usuario, 2026-09-21)</t>
         </is>
       </c>
       <c r="F10" t="n">
@@ -2676,12 +2676,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>comida por hora como mínimo por recolector (5 propio + 2,5 de medio acarreador); cumplida con margen: caza + frutos ≈ 10,0/h y pesca ≈ 8,6/h medidos en el mundo actual (semilla 12345)</t>
+          <t>comida por hora como mínimo por recolector (5 propio + 2,5 de medio acarreador); cumplida con margen: caza + frutos ≈ 12,2/h y pesca ≈ 8,6/h medidos en el mundo actual (semilla 12345)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Recoleccion.gd, balance del 2026-09-21 (caza 14 y frutos 8 por decisión del usuario)</t>
+          <t>Recoleccion.gd, balance del 2026-09-21 (caza 17 y frutos 10 por decisión del usuario)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: spec y plan de 2B, y hoja Extraccion del Excel
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Recursos.xlsx
+++ b/docs/Recursos.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relacion" sheetId="1" state="visible" r:id="rId1"/>
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Niveles" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Puestos" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Economia" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Extraccion" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -20,13 +21,18 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
@@ -52,15 +58,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -516,64 +526,64 @@
   <dimension ref="A2:AQ21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col width="17.7109375" customWidth="1" style="2" min="1" max="1"/>
-    <col width="12.7109375" customWidth="1" style="2" min="2" max="2"/>
-    <col width="13.42578125" customWidth="1" style="2" min="3" max="3"/>
-    <col width="12.7109375" customWidth="1" style="2" min="4" max="7"/>
-    <col width="3.28515625" customWidth="1" style="2" min="9" max="9"/>
-    <col width="11.5703125" customWidth="1" style="2" min="10" max="13"/>
-    <col width="3.28515625" customWidth="1" style="2" min="14" max="14"/>
-    <col width="12.85546875" customWidth="1" style="2" min="20" max="20"/>
-    <col width="2.5703125" customWidth="1" style="2" min="29" max="29"/>
+    <col width="17.7109375" customWidth="1" style="3" min="1" max="1"/>
+    <col width="12.7109375" customWidth="1" style="3" min="2" max="2"/>
+    <col width="13.42578125" customWidth="1" style="3" min="3" max="3"/>
+    <col width="12.7109375" customWidth="1" style="3" min="4" max="7"/>
+    <col width="3.28515625" customWidth="1" style="3" min="9" max="9"/>
+    <col width="11.5703125" customWidth="1" style="3" min="10" max="13"/>
+    <col width="3.28515625" customWidth="1" style="3" min="14" max="14"/>
+    <col width="12.85546875" customWidth="1" style="3" min="20" max="20"/>
+    <col width="2.5703125" customWidth="1" style="3" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="2">
-      <c r="B2" s="1" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Consumo por Tipo de unidad</t>
         </is>
       </c>
-      <c r="J2" s="1" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Consumo por Objeto</t>
         </is>
       </c>
-      <c r="O2" s="1" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>Costo/producción por Bloque o NPC</t>
         </is>
       </c>
-      <c r="AD2" s="1" t="inlineStr">
+      <c r="AD2" s="2" t="inlineStr">
         <is>
           <t>Siderúrgica</t>
         </is>
       </c>
-      <c r="AF2" s="1" t="inlineStr">
+      <c r="AF2" s="2" t="inlineStr">
         <is>
           <t>Refinería de mineral</t>
         </is>
       </c>
-      <c r="AH2" s="1" t="inlineStr">
+      <c r="AH2" s="2" t="inlineStr">
         <is>
           <t>Aserradero</t>
         </is>
       </c>
-      <c r="AJ2" s="1" t="inlineStr">
+      <c r="AJ2" s="2" t="inlineStr">
         <is>
           <t>Carbonera</t>
         </is>
       </c>
-      <c r="AL2" s="1" t="inlineStr">
+      <c r="AL2" s="2" t="inlineStr">
         <is>
           <t>Refinería petrolera</t>
         </is>
       </c>
-      <c r="AN2" s="1" t="inlineStr">
+      <c r="AN2" s="2" t="inlineStr">
         <is>
           <t>Licuefacftora de hidrocarburo</t>
         </is>
       </c>
-      <c r="AP2" s="1" t="inlineStr">
+      <c r="AP2" s="2" t="inlineStr">
         <is>
           <t>Central termoeléctrica</t>
         </is>
@@ -796,7 +806,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6">
@@ -806,7 +816,7 @@
         </is>
       </c>
       <c r="Q6" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="AD6" t="n">
         <v>2</v>
@@ -829,7 +839,7 @@
         </is>
       </c>
       <c r="R8" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9">
@@ -839,7 +849,7 @@
         </is>
       </c>
       <c r="S9" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="AK9" t="n">
         <v>1</v>
@@ -858,7 +868,7 @@
         </is>
       </c>
       <c r="T10" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="AF10" t="n">
         <v>3</v>
@@ -941,7 +951,7 @@
         <v>1</v>
       </c>
       <c r="O15" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="AH15" t="n">
         <v>1</v>
@@ -1159,12 +1169,12 @@
   <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="26.140625" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
-    <col width="33.140625" customWidth="1" style="2" min="2" max="2"/>
-    <col width="16.140625" bestFit="1" customWidth="1" style="2" min="3" max="3"/>
-    <col width="17" bestFit="1" customWidth="1" style="2" min="4" max="4"/>
-    <col width="31.5703125" bestFit="1" customWidth="1" style="2" min="5" max="5"/>
-    <col width="58.42578125" bestFit="1" customWidth="1" style="2" min="6" max="6"/>
+    <col width="26.140625" bestFit="1" customWidth="1" style="3" min="1" max="1"/>
+    <col width="33.140625" customWidth="1" style="3" min="2" max="2"/>
+    <col width="16.140625" bestFit="1" customWidth="1" style="3" min="3" max="3"/>
+    <col width="17" bestFit="1" customWidth="1" style="3" min="4" max="4"/>
+    <col width="31.5703125" bestFit="1" customWidth="1" style="3" min="5" max="5"/>
+    <col width="58.42578125" bestFit="1" customWidth="1" style="3" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1431,12 +1441,12 @@
   <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="43.28515625" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
-    <col width="34.28515625" bestFit="1" customWidth="1" style="2" min="2" max="2"/>
-    <col width="40.28515625" bestFit="1" customWidth="1" style="2" min="3" max="3"/>
-    <col width="24.85546875" bestFit="1" customWidth="1" style="2" min="4" max="4"/>
-    <col width="26.140625" bestFit="1" customWidth="1" style="2" min="5" max="5"/>
-    <col width="36.28515625" bestFit="1" customWidth="1" style="2" min="6" max="6"/>
+    <col width="43.28515625" bestFit="1" customWidth="1" style="3" min="1" max="1"/>
+    <col width="34.28515625" bestFit="1" customWidth="1" style="3" min="2" max="2"/>
+    <col width="40.28515625" bestFit="1" customWidth="1" style="3" min="3" max="3"/>
+    <col width="24.85546875" bestFit="1" customWidth="1" style="3" min="4" max="4"/>
+    <col width="26.140625" bestFit="1" customWidth="1" style="3" min="5" max="5"/>
+    <col width="36.28515625" bestFit="1" customWidth="1" style="3" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1605,73 +1615,72 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" style="2" min="1" max="1"/>
-    <col width="14" customWidth="1" style="2" min="2" max="2"/>
-    <col width="20" customWidth="1" style="2" min="3" max="3"/>
-    <col width="18" customWidth="1" style="2" min="4" max="4"/>
-    <col width="46" customWidth="1" style="2" min="5" max="5"/>
-    <col width="12" customWidth="1" style="2" min="6" max="6"/>
-    <col width="12" customWidth="1" style="2" min="7" max="7"/>
-    <col width="16" customWidth="1" style="2" min="8" max="8"/>
-    <col width="30" customWidth="1" style="2" min="9" max="9"/>
-    <col width="32" customWidth="1" style="2" min="10" max="10"/>
-    <col width="34" customWidth="1" style="2" min="11" max="11"/>
+    <col width="24" customWidth="1" style="3" min="1" max="1"/>
+    <col width="14" customWidth="1" style="3" min="2" max="2"/>
+    <col width="20" customWidth="1" style="3" min="3" max="3"/>
+    <col width="18" customWidth="1" style="3" min="4" max="4"/>
+    <col width="46" customWidth="1" style="3" min="5" max="5"/>
+    <col width="12" customWidth="1" style="3" min="6" max="7"/>
+    <col width="16" customWidth="1" style="3" min="8" max="8"/>
+    <col width="30" customWidth="1" style="3" min="9" max="9"/>
+    <col width="32" customWidth="1" style="3" min="10" max="10"/>
+    <col width="34" customWidth="1" style="3" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+    <row r="1" ht="45" customHeight="1" s="3">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Puesto</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Clave de tasa</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Recurso en el almacén</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Tasa base (unid/trabajador/hora)</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Se multiplica por</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Personal máximo</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Almacén local</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Huella (ancho x alto)</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Radio del área</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
@@ -2415,31 +2424,31 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="52" customWidth="1" style="2" min="1" max="1"/>
-    <col width="10" customWidth="1" style="2" min="2" max="2"/>
-    <col width="62" customWidth="1" style="2" min="3" max="3"/>
-    <col width="40" customWidth="1" style="2" min="4" max="4"/>
+    <col width="52" customWidth="1" style="3" min="1" max="1"/>
+    <col width="10" customWidth="1" style="3" min="2" max="2"/>
+    <col width="62" customWidth="1" style="3" min="3" max="3"/>
+    <col width="40" customWidth="1" style="3" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Parámetro</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Valor</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Unidad</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
@@ -2762,6 +2771,396 @@
       <c r="D17" t="inlineStr">
         <is>
           <t>Recoleccion.ESCALA_AGUA_MAX</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" style="3" min="1" max="1"/>
+    <col width="34" customWidth="1" style="3" min="2" max="2"/>
+    <col width="16" customWidth="1" style="3" min="3" max="3"/>
+    <col width="28" customWidth="1" style="3" min="4" max="4"/>
+    <col width="16" customWidth="1" style="3" min="5" max="5"/>
+    <col width="44" customWidth="1" style="3" min="6" max="6"/>
+    <col width="52" customWidth="1" style="3" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Recurso</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Bloque de extracción</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Unidades por bloque extraído</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Bloque de construcción que lo consume</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Unidades por bloque construido</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Nota</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>tierra</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>tierra (incluye la capa piso)</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>tierra</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Extracción: decidido 2026-09-24. Construcción: propuesta</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>1-1-1 a propósito, para no crear "tierra de construcción"</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>piedra</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>piedra</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>10</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>pared, piso, etc.</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Extracción: decidido 2026-09-24. Construcción: propuesta (ejemplo, sin cobrar todavía)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Ejemplo: minar 1 bloque da 10 de piedra; colocar 1 pared cuesta 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>hierro</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>hierro</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>10</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>por definir</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Extracción: decidido 2026-09-24</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>cobre</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>cobre</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>por definir</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Extracción: decidido 2026-09-24</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>carbon</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>carbón</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>por definir</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Extracción: decidido 2026-09-24</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>tierras_raras</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>tierras raras</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>10</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>por definir</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Extracción: decidido 2026-09-24</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>madera</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>tronco (por celda de tronco; el follaje no rinde)</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>por definir</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Extracción: decidido 2026-09-24</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>La salud de un árbol es su cantidad de celdas de tronco</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>agua</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>agua</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Reservado (sin uso en 2B)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Antes 2 por bloque en la hoja Relacion</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>crudo</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>petróleo</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Reservado (sin uso en 2B)</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>No existe en el mundo todavía (fluidos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Modelo de tres capas</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>1. Extracción: se retira un bloque de extracción del mundo (por el avatar o por un puesto) y rinde las unidades de la columna C.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2. Unidad de recurso: lo que se guarda en el almacén (inventario del avatar = almacén central de la ciudad).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>3. Construcción: colocar un bloque de construcción consume unidades del almacén (columna E). Aún no se cobra; la hoja lo deja definido para cuando exista.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Sustituye el 5 por bloque de la hoja Relacion (columnas O a T): ahora 10 para sólidos, 1 para tierra y 2 para líquidos.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: documentar la extracción física y el agotamiento (2B)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Recursos.xlsx
+++ b/docs/Recursos.xlsx
@@ -2423,7 +2423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" style="3" min="1" max="1"/>
@@ -2537,20 +2537,20 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Límite del stock central</t>
+          <t>Límite del stock central (inventario del avatar)</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>unidades por recurso (comida: 10000)</t>
+          <t>unidades por recurso al inicio (comida: 5000); ×2 al declarar el núcleo; +100 por baúl (comida +400) de cada edificio residencial posterior al núcleo</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Ciudad.almacen</t>
+          <t>Ciudad.LIMITE_BASE / LIMITE_BASE_COMIDA / FACTOR_NUCLEO / BONO_BAUL / BONO_BAUL_COMIDA</t>
         </is>
       </c>
     </row>
@@ -2561,16 +2561,16 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>10000</v>
+        <v>1500</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>unidades (al máximo)</t>
+          <t>unidades (300 ticks de un avatar sin producción)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Ciudad.almacen</t>
+          <t>Ciudad.COMIDA_INICIAL</t>
         </is>
       </c>
     </row>
@@ -2771,6 +2771,126 @@
       <c r="D17" t="inlineStr">
         <is>
           <t>Recoleccion.ESCALA_AGUA_MAX</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Ticks entre recálculos de tasas</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>6</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>horas de juego</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Economia.TICKS_RECALCULO</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Profundidad mínima de extracción de una mina</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>bloques bajo la superficie natural (GROSOR_TIERRA - 2)</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Recoleccion.PROFUNDIDAD_MINIMA_EXTRACCION</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Comida por recolección de frutos (a densidad 1.0)</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>60</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>unidades; el árbol no se consume</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Recoleccion.COMIDA_POR_RECOLECCION</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Rebrote de frutos</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>24</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>horas de juego</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Recoleccion.HORAS_REBROTE_FRUTOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Tiempo de recolección de frutos</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>2</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>segundos</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Recoleccion.TIEMPO_RECOLECCION_FRUTOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Tiempo de tala por punto de salud</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>segundos</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Recoleccion.TIEMPO_TALA_POR_SALUD</t>
         </is>
       </c>
     </row>
@@ -2929,7 +3049,6 @@
           <t>Extracción: decidido 2026-09-24</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2960,7 +3079,6 @@
           <t>Extracción: decidido 2026-09-24</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2991,7 +3109,6 @@
           <t>Extracción: decidido 2026-09-24</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3022,7 +3139,6 @@
           <t>Extracción: decidido 2026-09-24</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">

</xml_diff>

<commit_message>
docs: fichas de extracción, balance de población y decisión de reembolso al minar
Fichas_Consumo_Produccion.md: añade la tabla de bloques minables →
unidades de recurso → bloques colocables (hoja "Extraccion" del Excel),
corrige la sección 1 según el balance 2026-09-28 (Ciudadano x_cama 5,
Especialista sin combustible, Militar combustible 2) y quita una nota
desactualizada sobre extracción física (ya implementada en 2B).

Recursos.xlsx: hoja "Relacion" actualizada al mismo balance.

Pendientes y próximos pasos.md / spec de extracción 2B: documentan la
decisión de que volver a minar un bloque colocado por el jugador
reembolse su costo de colocación, para cuando el sub-proyecto 2C
implemente el cobro de construcción.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Recursos.xlsx
+++ b/docs/Recursos.xlsx
@@ -523,7 +523,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:AQ21"/>
+  <dimension ref="A1:AQ21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="17.7109375" customWidth="1" style="3" min="1" max="1"/>
@@ -537,6 +537,7 @@
     <col width="2.5703125" customWidth="1" style="3" min="29" max="29"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="2" t="inlineStr">
         <is>
@@ -919,11 +920,8 @@
           <t>Combustible</t>
         </is>
       </c>
-      <c r="F14" t="n">
-        <v>1</v>
-      </c>
       <c r="H14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AM14" t="n">
         <v>1</v>
@@ -1035,7 +1033,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C18" t="n">
         <v>4</v>

</xml_diff>